<commit_message>
update dashboard data 2026-06-26 14:53
</commit_message>
<xml_diff>
--- a/docs/reports/NCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
+++ b/docs/reports/NCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
@@ -9824,7 +9824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -9843,6 +9843,7 @@
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="46" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9942,6 +9943,11 @@
           <t>Suspected Reason (undesirable)</t>
         </is>
       </c>
+      <c r="Q5" s="14" t="inlineStr">
+        <is>
+          <t>Loco Type</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="49" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -10017,6 +10023,11 @@
           <t>PG issue (speed fluctuation)</t>
         </is>
       </c>
+      <c r="Q6" s="31" t="inlineStr">
+        <is>
+          <t>HBL</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
@@ -10078,7 +10089,7 @@
       </c>
       <c r="N7" s="36" t="inlineStr">
         <is>
-          <t>6924</t>
+          <t>2952</t>
         </is>
       </c>
       <c r="O7" s="16" t="inlineStr">
@@ -10089,6 +10100,11 @@
       <c r="P7" s="34" t="inlineStr">
         <is>
           <t>FS-&gt;SR degradation + EB</t>
+        </is>
+      </c>
+      <c r="Q7" s="16" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
         </is>
       </c>
     </row>
@@ -10165,6 +10181,11 @@
           <t>Trip mode</t>
         </is>
       </c>
+      <c r="Q8" s="16" t="inlineStr">
+        <is>
+          <t>HBL</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -10239,6 +10260,11 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
+      <c r="Q9" s="16" t="inlineStr">
+        <is>
+          <t>HBL</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -10313,6 +10339,11 @@
           <t>FS-&gt;SR degradation + EB</t>
         </is>
       </c>
+      <c r="Q10" s="16" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -10387,11 +10418,16 @@
           <t>Trip mode</t>
         </is>
       </c>
+      <c r="Q11" s="16" t="inlineStr">
+        <is>
+          <t>HBL</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update NCR dashboard data
</commit_message>
<xml_diff>
--- a/docs/reports/NCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
+++ b/docs/reports/NCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="#,##0.0"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.00000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -184,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -206,13 +206,13 @@
     <xf numFmtId="3" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -228,7 +228,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -258,7 +258,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -302,6 +302,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,7 +725,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -850,19 +867,19 @@
         <f>'Daily Breakdown'!J222</f>
         <v/>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="44">
         <f>IFERROR(G5/D5,0)</f>
         <v/>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="45">
         <f>IFERROR(G5/E5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="46">
         <f>IFERROR(G5/E5*100,0)</f>
         <v/>
       </c>
-      <c r="M5" s="10">
+      <c r="M5" s="45">
         <f>IFERROR(G5/(D5*E5/1000),0)</f>
         <v/>
       </c>
@@ -870,19 +887,19 @@
         <f>'Daily Breakdown'!K222</f>
         <v/>
       </c>
-      <c r="O5" s="9">
+      <c r="O5" s="44">
         <f>IFERROR(N5/D5,0)</f>
         <v/>
       </c>
-      <c r="P5" s="10">
+      <c r="P5" s="45">
         <f>IFERROR(N5/E5,0)</f>
         <v/>
       </c>
-      <c r="Q5" s="10">
+      <c r="Q5" s="45">
         <f>IFERROR(N5/(D5*E5/100),0)</f>
         <v/>
       </c>
-      <c r="R5" s="11">
+      <c r="R5" s="46">
         <f>IFERROR(N5/E5*100,0)</f>
         <v/>
       </c>
@@ -932,7 +949,13 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" s="37" t="inlineStr">
+        <is>
+          <t>Availability base excludes locos with FS+OS pkts = 0 (they are still listed; only the Total-pkts availability base drops them).</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -1004,7 +1027,7 @@
       <c r="C4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="17" t="n">
+      <c r="D4" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E4" s="18" t="n">
@@ -1044,7 +1067,7 @@
       <c r="C5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E5" s="18" t="n">
@@ -1084,7 +1107,7 @@
       <c r="C6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E6" s="18" t="n">
@@ -1124,7 +1147,7 @@
       <c r="C7" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E7" s="18" t="n">
@@ -1164,7 +1187,7 @@
       <c r="C8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E8" s="18" t="n">
@@ -1204,7 +1227,7 @@
       <c r="C9" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E9" s="18" t="n">
@@ -1244,7 +1267,7 @@
       <c r="C10" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E10" s="18" t="n">
@@ -1284,7 +1307,7 @@
       <c r="C11" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E11" s="18" t="n">
@@ -1324,7 +1347,7 @@
       <c r="C12" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="47" t="n">
         <v>77.76000000000001</v>
       </c>
       <c r="E12" s="18" t="n">
@@ -1364,7 +1387,7 @@
       <c r="C13" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="47" t="n">
         <v>77.16</v>
       </c>
       <c r="E13" s="18" t="n">
@@ -1404,7 +1427,7 @@
       <c r="C14" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="47" t="n">
         <v>74.55</v>
       </c>
       <c r="E14" s="18" t="n">
@@ -1444,7 +1467,7 @@
       <c r="C15" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="47" t="n">
         <v>77.67</v>
       </c>
       <c r="E15" s="18" t="n">
@@ -1484,7 +1507,7 @@
       <c r="C16" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="47" t="n">
         <v>77.73</v>
       </c>
       <c r="E16" s="18" t="n">
@@ -1524,7 +1547,7 @@
       <c r="C17" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="D17" s="47" t="n">
         <v>77.73999999999999</v>
       </c>
       <c r="E17" s="18" t="n">
@@ -1564,7 +1587,7 @@
       <c r="C18" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="47" t="n">
         <v>77.64</v>
       </c>
       <c r="E18" s="18" t="n">
@@ -1604,7 +1627,7 @@
       <c r="C19" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="D19" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E19" s="18" t="n">
@@ -1644,7 +1667,7 @@
       <c r="C20" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="47" t="n">
         <v>76.90000000000001</v>
       </c>
       <c r="E20" s="18" t="n">
@@ -1684,7 +1707,7 @@
       <c r="C21" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="D21" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E21" s="18" t="n">
@@ -1724,7 +1747,7 @@
       <c r="C22" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E22" s="18" t="n">
@@ -1764,7 +1787,7 @@
       <c r="C23" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="D23" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E23" s="18" t="n">
@@ -1804,7 +1827,7 @@
       <c r="C24" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E24" s="18" t="n">
@@ -1844,7 +1867,7 @@
       <c r="C25" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="17" t="n">
+      <c r="D25" s="47" t="n">
         <v>77.8</v>
       </c>
       <c r="E25" s="18" t="n">
@@ -1884,7 +1907,7 @@
       <c r="C26" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="47" t="n">
         <v>77.70999999999999</v>
       </c>
       <c r="E26" s="18" t="n">
@@ -1924,7 +1947,7 @@
       <c r="C27" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E27" s="18" t="n">
@@ -1964,7 +1987,7 @@
       <c r="C28" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="47" t="n">
         <v>77.67</v>
       </c>
       <c r="E28" s="18" t="n">
@@ -2004,7 +2027,7 @@
       <c r="C29" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="47" t="n">
         <v>77.64</v>
       </c>
       <c r="E29" s="18" t="n">
@@ -2044,7 +2067,7 @@
       <c r="C30" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="47" t="n">
         <v>77.67</v>
       </c>
       <c r="E30" s="18" t="n">
@@ -2084,7 +2107,7 @@
       <c r="C31" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="17" t="n">
+      <c r="D31" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E31" s="18" t="n">
@@ -2124,7 +2147,7 @@
       <c r="C32" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="17" t="n">
+      <c r="D32" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E32" s="18" t="n">
@@ -2164,7 +2187,7 @@
       <c r="C33" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="17" t="n">
+      <c r="D33" s="47" t="n">
         <v>77.70999999999999</v>
       </c>
       <c r="E33" s="18" t="n">
@@ -2204,7 +2227,7 @@
       <c r="C34" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="17" t="n">
+      <c r="D34" s="47" t="n">
         <v>3.76</v>
       </c>
       <c r="E34" s="18" t="n">
@@ -2245,7 +2268,7 @@
         <f>SUM(C4:C34)</f>
         <v/>
       </c>
-      <c r="D35" s="22">
+      <c r="D35" s="48">
         <f>SUM(D4:D34)</f>
         <v/>
       </c>
@@ -2254,7 +2277,7 @@
         <v/>
       </c>
       <c r="F35" s="23">
-        <f>SUM(F4:F34)</f>
+        <f>SUMIF(E4:E34,"&gt;0",F4:F34)</f>
         <v/>
       </c>
       <c r="G35" s="24">
@@ -2292,7 +2315,7 @@
       <c r="C36" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D36" s="17" t="n">
+      <c r="D36" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E36" s="18" t="n">
@@ -2332,7 +2355,7 @@
       <c r="C37" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D37" s="17" t="n">
+      <c r="D37" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E37" s="18" t="n">
@@ -2372,7 +2395,7 @@
       <c r="C38" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D38" s="17" t="n">
+      <c r="D38" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E38" s="18" t="n">
@@ -2412,7 +2435,7 @@
       <c r="C39" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="17" t="n">
+      <c r="D39" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E39" s="18" t="n">
@@ -2452,7 +2475,7 @@
       <c r="C40" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D40" s="17" t="n">
+      <c r="D40" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E40" s="18" t="n">
@@ -2492,7 +2515,7 @@
       <c r="C41" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="17" t="n">
+      <c r="D41" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E41" s="18" t="n">
@@ -2532,7 +2555,7 @@
       <c r="C42" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D42" s="17" t="n">
+      <c r="D42" s="47" t="n">
         <v>60.51</v>
       </c>
       <c r="E42" s="18" t="n">
@@ -2572,7 +2595,7 @@
       <c r="C43" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D43" s="17" t="n">
+      <c r="D43" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E43" s="18" t="n">
@@ -2612,7 +2635,7 @@
       <c r="C44" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="17" t="n">
+      <c r="D44" s="47" t="n">
         <v>77.66</v>
       </c>
       <c r="E44" s="18" t="n">
@@ -2652,7 +2675,7 @@
       <c r="C45" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="17" t="n">
+      <c r="D45" s="47" t="n">
         <v>77.68000000000001</v>
       </c>
       <c r="E45" s="18" t="n">
@@ -2692,7 +2715,7 @@
       <c r="C46" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D46" s="17" t="n">
+      <c r="D46" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E46" s="18" t="n">
@@ -2732,7 +2755,7 @@
       <c r="C47" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D47" s="17" t="n">
+      <c r="D47" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E47" s="18" t="n">
@@ -2772,7 +2795,7 @@
       <c r="C48" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="17" t="n">
+      <c r="D48" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E48" s="18" t="n">
@@ -2812,7 +2835,7 @@
       <c r="C49" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D49" s="17" t="n">
+      <c r="D49" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E49" s="18" t="n">
@@ -2852,7 +2875,7 @@
       <c r="C50" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D50" s="17" t="n">
+      <c r="D50" s="47" t="n">
         <v>77.67</v>
       </c>
       <c r="E50" s="18" t="n">
@@ -2892,7 +2915,7 @@
       <c r="C51" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D51" s="17" t="n">
+      <c r="D51" s="47" t="n">
         <v>77.79000000000001</v>
       </c>
       <c r="E51" s="18" t="n">
@@ -2932,7 +2955,7 @@
       <c r="C52" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D52" s="17" t="n">
+      <c r="D52" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E52" s="18" t="n">
@@ -2972,7 +2995,7 @@
       <c r="C53" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D53" s="17" t="n">
+      <c r="D53" s="47" t="n">
         <v>77.73</v>
       </c>
       <c r="E53" s="18" t="n">
@@ -3012,7 +3035,7 @@
       <c r="C54" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D54" s="17" t="n">
+      <c r="D54" s="47" t="n">
         <v>77.66</v>
       </c>
       <c r="E54" s="18" t="n">
@@ -3052,7 +3075,7 @@
       <c r="C55" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D55" s="17" t="n">
+      <c r="D55" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E55" s="18" t="n">
@@ -3092,7 +3115,7 @@
       <c r="C56" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D56" s="17" t="n">
+      <c r="D56" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E56" s="18" t="n">
@@ -3132,7 +3155,7 @@
       <c r="C57" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D57" s="17" t="n">
+      <c r="D57" s="47" t="n">
         <v>77.81999999999999</v>
       </c>
       <c r="E57" s="18" t="n">
@@ -3172,7 +3195,7 @@
       <c r="C58" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D58" s="17" t="n">
+      <c r="D58" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E58" s="18" t="n">
@@ -3212,7 +3235,7 @@
       <c r="C59" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D59" s="17" t="n">
+      <c r="D59" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E59" s="18" t="n">
@@ -3252,7 +3275,7 @@
       <c r="C60" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D60" s="17" t="n">
+      <c r="D60" s="47" t="n">
         <v>77.73999999999999</v>
       </c>
       <c r="E60" s="18" t="n">
@@ -3292,7 +3315,7 @@
       <c r="C61" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D61" s="17" t="n">
+      <c r="D61" s="47" t="n">
         <v>70.48</v>
       </c>
       <c r="E61" s="18" t="n">
@@ -3332,7 +3355,7 @@
       <c r="C62" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D62" s="17" t="n">
+      <c r="D62" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E62" s="18" t="n">
@@ -3372,7 +3395,7 @@
       <c r="C63" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D63" s="17" t="n">
+      <c r="D63" s="47" t="n">
         <v>18.89</v>
       </c>
       <c r="E63" s="18" t="n">
@@ -3412,7 +3435,7 @@
       <c r="C64" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D64" s="17" t="n">
+      <c r="D64" s="47" t="n">
         <v>7.02</v>
       </c>
       <c r="E64" s="18" t="n">
@@ -3453,7 +3476,7 @@
         <f>SUM(C36:C64)</f>
         <v/>
       </c>
-      <c r="D65" s="22">
+      <c r="D65" s="48">
         <f>SUM(D36:D64)</f>
         <v/>
       </c>
@@ -3462,7 +3485,7 @@
         <v/>
       </c>
       <c r="F65" s="23">
-        <f>SUM(F36:F64)</f>
+        <f>SUMIF(E36:E64,"&gt;0",F36:F64)</f>
         <v/>
       </c>
       <c r="G65" s="24">
@@ -3500,7 +3523,7 @@
       <c r="C66" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D66" s="17" t="n">
+      <c r="D66" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E66" s="18" t="n">
@@ -3540,7 +3563,7 @@
       <c r="C67" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D67" s="17" t="n">
+      <c r="D67" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E67" s="18" t="n">
@@ -3580,7 +3603,7 @@
       <c r="C68" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D68" s="17" t="n">
+      <c r="D68" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E68" s="18" t="n">
@@ -3620,7 +3643,7 @@
       <c r="C69" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D69" s="17" t="n">
+      <c r="D69" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E69" s="18" t="n">
@@ -3660,7 +3683,7 @@
       <c r="C70" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D70" s="17" t="n">
+      <c r="D70" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E70" s="18" t="n">
@@ -3700,7 +3723,7 @@
       <c r="C71" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D71" s="17" t="n">
+      <c r="D71" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E71" s="18" t="n">
@@ -3740,7 +3763,7 @@
       <c r="C72" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D72" s="17" t="n">
+      <c r="D72" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E72" s="18" t="n">
@@ -3780,7 +3803,7 @@
       <c r="C73" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D73" s="17" t="n">
+      <c r="D73" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E73" s="18" t="n">
@@ -3820,7 +3843,7 @@
       <c r="C74" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D74" s="17" t="n">
+      <c r="D74" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E74" s="18" t="n">
@@ -3860,7 +3883,7 @@
       <c r="C75" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D75" s="17" t="n">
+      <c r="D75" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E75" s="18" t="n">
@@ -3900,7 +3923,7 @@
       <c r="C76" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D76" s="17" t="n">
+      <c r="D76" s="47" t="n">
         <v>77.63</v>
       </c>
       <c r="E76" s="18" t="n">
@@ -3940,7 +3963,7 @@
       <c r="C77" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D77" s="17" t="n">
+      <c r="D77" s="47" t="n">
         <v>77.75</v>
       </c>
       <c r="E77" s="18" t="n">
@@ -3980,7 +4003,7 @@
       <c r="C78" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D78" s="17" t="n">
+      <c r="D78" s="47" t="n">
         <v>77.81</v>
       </c>
       <c r="E78" s="18" t="n">
@@ -4020,7 +4043,7 @@
       <c r="C79" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D79" s="17" t="n">
+      <c r="D79" s="47" t="n">
         <v>77.73</v>
       </c>
       <c r="E79" s="18" t="n">
@@ -4060,7 +4083,7 @@
       <c r="C80" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D80" s="17" t="n">
+      <c r="D80" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E80" s="18" t="n">
@@ -4100,7 +4123,7 @@
       <c r="C81" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D81" s="17" t="n">
+      <c r="D81" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E81" s="18" t="n">
@@ -4140,7 +4163,7 @@
       <c r="C82" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D82" s="17" t="n">
+      <c r="D82" s="47" t="n">
         <v>77.67</v>
       </c>
       <c r="E82" s="18" t="n">
@@ -4180,7 +4203,7 @@
       <c r="C83" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D83" s="17" t="n">
+      <c r="D83" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E83" s="18" t="n">
@@ -4220,7 +4243,7 @@
       <c r="C84" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D84" s="17" t="n">
+      <c r="D84" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E84" s="18" t="n">
@@ -4260,7 +4283,7 @@
       <c r="C85" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D85" s="17" t="n">
+      <c r="D85" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E85" s="18" t="n">
@@ -4300,7 +4323,7 @@
       <c r="C86" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D86" s="17" t="n">
+      <c r="D86" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E86" s="18" t="n">
@@ -4340,7 +4363,7 @@
       <c r="C87" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D87" s="17" t="n">
+      <c r="D87" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E87" s="18" t="n">
@@ -4380,7 +4403,7 @@
       <c r="C88" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D88" s="17" t="n">
+      <c r="D88" s="47" t="n">
         <v>77.58</v>
       </c>
       <c r="E88" s="18" t="n">
@@ -4420,7 +4443,7 @@
       <c r="C89" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D89" s="17" t="n">
+      <c r="D89" s="47" t="n">
         <v>77.73999999999999</v>
       </c>
       <c r="E89" s="18" t="n">
@@ -4460,7 +4483,7 @@
       <c r="C90" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D90" s="17" t="n">
+      <c r="D90" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E90" s="18" t="n">
@@ -4500,7 +4523,7 @@
       <c r="C91" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D91" s="17" t="n">
+      <c r="D91" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E91" s="18" t="n">
@@ -4540,7 +4563,7 @@
       <c r="C92" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D92" s="17" t="n">
+      <c r="D92" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E92" s="18" t="n">
@@ -4580,7 +4603,7 @@
       <c r="C93" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D93" s="17" t="n">
+      <c r="D93" s="47" t="n">
         <v>7.27</v>
       </c>
       <c r="E93" s="18" t="n">
@@ -4620,7 +4643,7 @@
       <c r="C94" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D94" s="17" t="n">
+      <c r="D94" s="47" t="n">
         <v>2.56</v>
       </c>
       <c r="E94" s="18" t="n">
@@ -4661,7 +4684,7 @@
         <f>SUM(C66:C94)</f>
         <v/>
       </c>
-      <c r="D95" s="22">
+      <c r="D95" s="48">
         <f>SUM(D66:D94)</f>
         <v/>
       </c>
@@ -4670,7 +4693,7 @@
         <v/>
       </c>
       <c r="F95" s="23">
-        <f>SUM(F66:F94)</f>
+        <f>SUMIF(E66:E94,"&gt;0",F66:F94)</f>
         <v/>
       </c>
       <c r="G95" s="24">
@@ -4708,7 +4731,7 @@
       <c r="C96" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D96" s="17" t="n">
+      <c r="D96" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E96" s="18" t="n">
@@ -4748,7 +4771,7 @@
       <c r="C97" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D97" s="17" t="n">
+      <c r="D97" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E97" s="18" t="n">
@@ -4788,7 +4811,7 @@
       <c r="C98" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D98" s="17" t="n">
+      <c r="D98" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E98" s="18" t="n">
@@ -4828,7 +4851,7 @@
       <c r="C99" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D99" s="17" t="n">
+      <c r="D99" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E99" s="18" t="n">
@@ -4868,7 +4891,7 @@
       <c r="C100" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D100" s="17" t="n">
+      <c r="D100" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E100" s="18" t="n">
@@ -4908,7 +4931,7 @@
       <c r="C101" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D101" s="17" t="n">
+      <c r="D101" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E101" s="18" t="n">
@@ -4948,7 +4971,7 @@
       <c r="C102" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D102" s="17" t="n">
+      <c r="D102" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E102" s="18" t="n">
@@ -4988,7 +5011,7 @@
       <c r="C103" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D103" s="17" t="n">
+      <c r="D103" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E103" s="18" t="n">
@@ -5028,7 +5051,7 @@
       <c r="C104" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D104" s="17" t="n">
+      <c r="D104" s="47" t="n">
         <v>77.68000000000001</v>
       </c>
       <c r="E104" s="18" t="n">
@@ -5068,7 +5091,7 @@
       <c r="C105" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D105" s="17" t="n">
+      <c r="D105" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E105" s="18" t="n">
@@ -5108,7 +5131,7 @@
       <c r="C106" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D106" s="17" t="n">
+      <c r="D106" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E106" s="18" t="n">
@@ -5148,7 +5171,7 @@
       <c r="C107" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D107" s="17" t="n">
+      <c r="D107" s="47" t="n">
         <v>77.68000000000001</v>
       </c>
       <c r="E107" s="18" t="n">
@@ -5188,7 +5211,7 @@
       <c r="C108" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D108" s="17" t="n">
+      <c r="D108" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E108" s="18" t="n">
@@ -5228,7 +5251,7 @@
       <c r="C109" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D109" s="17" t="n">
+      <c r="D109" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E109" s="18" t="n">
@@ -5268,7 +5291,7 @@
       <c r="C110" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D110" s="17" t="n">
+      <c r="D110" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E110" s="18" t="n">
@@ -5308,7 +5331,7 @@
       <c r="C111" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D111" s="17" t="n">
+      <c r="D111" s="47" t="n">
         <v>77.59</v>
       </c>
       <c r="E111" s="18" t="n">
@@ -5348,7 +5371,7 @@
       <c r="C112" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D112" s="17" t="n">
+      <c r="D112" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E112" s="18" t="n">
@@ -5388,7 +5411,7 @@
       <c r="C113" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D113" s="17" t="n">
+      <c r="D113" s="47" t="n">
         <v>19.18</v>
       </c>
       <c r="E113" s="18" t="n">
@@ -5428,7 +5451,7 @@
       <c r="C114" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D114" s="17" t="n">
+      <c r="D114" s="47" t="n">
         <v>77.70999999999999</v>
       </c>
       <c r="E114" s="18" t="n">
@@ -5468,7 +5491,7 @@
       <c r="C115" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D115" s="17" t="n">
+      <c r="D115" s="47" t="n">
         <v>27.78</v>
       </c>
       <c r="E115" s="18" t="n">
@@ -5508,7 +5531,7 @@
       <c r="C116" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D116" s="17" t="n">
+      <c r="D116" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E116" s="18" t="n">
@@ -5548,7 +5571,7 @@
       <c r="C117" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D117" s="17" t="n">
+      <c r="D117" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E117" s="18" t="n">
@@ -5588,7 +5611,7 @@
       <c r="C118" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D118" s="17" t="n">
+      <c r="D118" s="47" t="n">
         <v>77.8</v>
       </c>
       <c r="E118" s="18" t="n">
@@ -5628,7 +5651,7 @@
       <c r="C119" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D119" s="17" t="n">
+      <c r="D119" s="47" t="n">
         <v>51.77</v>
       </c>
       <c r="E119" s="18" t="n">
@@ -5668,7 +5691,7 @@
       <c r="C120" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D120" s="17" t="n">
+      <c r="D120" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E120" s="18" t="n">
@@ -5708,7 +5731,7 @@
       <c r="C121" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D121" s="17" t="n">
+      <c r="D121" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E121" s="18" t="n">
@@ -5748,7 +5771,7 @@
       <c r="C122" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D122" s="17" t="n">
+      <c r="D122" s="47" t="n">
         <v>1.24</v>
       </c>
       <c r="E122" s="18" t="n">
@@ -5789,7 +5812,7 @@
         <f>SUM(C96:C122)</f>
         <v/>
       </c>
-      <c r="D123" s="22">
+      <c r="D123" s="48">
         <f>SUM(D96:D122)</f>
         <v/>
       </c>
@@ -5798,7 +5821,7 @@
         <v/>
       </c>
       <c r="F123" s="23">
-        <f>SUM(F96:F122)</f>
+        <f>SUMIF(E96:E122,"&gt;0",F96:F122)</f>
         <v/>
       </c>
       <c r="G123" s="24">
@@ -5836,7 +5859,7 @@
       <c r="C124" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D124" s="17" t="n">
+      <c r="D124" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E124" s="18" t="n">
@@ -5876,7 +5899,7 @@
       <c r="C125" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D125" s="17" t="n">
+      <c r="D125" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E125" s="18" t="n">
@@ -5916,7 +5939,7 @@
       <c r="C126" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D126" s="17" t="n">
+      <c r="D126" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E126" s="18" t="n">
@@ -5956,7 +5979,7 @@
       <c r="C127" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D127" s="17" t="n">
+      <c r="D127" s="47" t="n">
         <v>77.81999999999999</v>
       </c>
       <c r="E127" s="18" t="n">
@@ -5996,7 +6019,7 @@
       <c r="C128" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D128" s="17" t="n">
+      <c r="D128" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E128" s="18" t="n">
@@ -6036,7 +6059,7 @@
       <c r="C129" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D129" s="17" t="n">
+      <c r="D129" s="47" t="n">
         <v>77.70999999999999</v>
       </c>
       <c r="E129" s="18" t="n">
@@ -6076,7 +6099,7 @@
       <c r="C130" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D130" s="17" t="n">
+      <c r="D130" s="47" t="n">
         <v>77.73999999999999</v>
       </c>
       <c r="E130" s="18" t="n">
@@ -6116,7 +6139,7 @@
       <c r="C131" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D131" s="17" t="n">
+      <c r="D131" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E131" s="18" t="n">
@@ -6156,7 +6179,7 @@
       <c r="C132" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D132" s="17" t="n">
+      <c r="D132" s="47" t="n">
         <v>77.75</v>
       </c>
       <c r="E132" s="18" t="n">
@@ -6196,7 +6219,7 @@
       <c r="C133" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D133" s="17" t="n">
+      <c r="D133" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E133" s="18" t="n">
@@ -6236,7 +6259,7 @@
       <c r="C134" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D134" s="17" t="n">
+      <c r="D134" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E134" s="18" t="n">
@@ -6276,7 +6299,7 @@
       <c r="C135" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D135" s="17" t="n">
+      <c r="D135" s="47" t="n">
         <v>77.63</v>
       </c>
       <c r="E135" s="18" t="n">
@@ -6316,7 +6339,7 @@
       <c r="C136" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D136" s="17" t="n">
+      <c r="D136" s="47" t="n">
         <v>77.62</v>
       </c>
       <c r="E136" s="18" t="n">
@@ -6356,7 +6379,7 @@
       <c r="C137" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D137" s="17" t="n">
+      <c r="D137" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E137" s="18" t="n">
@@ -6396,7 +6419,7 @@
       <c r="C138" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D138" s="17" t="n">
+      <c r="D138" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E138" s="18" t="n">
@@ -6436,7 +6459,7 @@
       <c r="C139" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D139" s="17" t="n">
+      <c r="D139" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E139" s="18" t="n">
@@ -6476,7 +6499,7 @@
       <c r="C140" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D140" s="17" t="n">
+      <c r="D140" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E140" s="18" t="n">
@@ -6516,7 +6539,7 @@
       <c r="C141" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D141" s="17" t="n">
+      <c r="D141" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E141" s="18" t="n">
@@ -6556,7 +6579,7 @@
       <c r="C142" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D142" s="17" t="n">
+      <c r="D142" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E142" s="18" t="n">
@@ -6596,7 +6619,7 @@
       <c r="C143" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D143" s="17" t="n">
+      <c r="D143" s="47" t="n">
         <v>77.81</v>
       </c>
       <c r="E143" s="18" t="n">
@@ -6636,7 +6659,7 @@
       <c r="C144" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D144" s="17" t="n">
+      <c r="D144" s="47" t="n">
         <v>77.77</v>
       </c>
       <c r="E144" s="18" t="n">
@@ -6676,7 +6699,7 @@
       <c r="C145" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D145" s="17" t="n">
+      <c r="D145" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E145" s="18" t="n">
@@ -6716,7 +6739,7 @@
       <c r="C146" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D146" s="17" t="n">
+      <c r="D146" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E146" s="18" t="n">
@@ -6756,7 +6779,7 @@
       <c r="C147" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D147" s="17" t="n">
+      <c r="D147" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E147" s="18" t="n">
@@ -6796,7 +6819,7 @@
       <c r="C148" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D148" s="17" t="n">
+      <c r="D148" s="47" t="n">
         <v>77.8</v>
       </c>
       <c r="E148" s="18" t="n">
@@ -6836,7 +6859,7 @@
       <c r="C149" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D149" s="17" t="n">
+      <c r="D149" s="47" t="n">
         <v>8.59</v>
       </c>
       <c r="E149" s="18" t="n">
@@ -6877,7 +6900,7 @@
         <f>SUM(C124:C149)</f>
         <v/>
       </c>
-      <c r="D150" s="22">
+      <c r="D150" s="48">
         <f>SUM(D124:D149)</f>
         <v/>
       </c>
@@ -6886,7 +6909,7 @@
         <v/>
       </c>
       <c r="F150" s="23">
-        <f>SUM(F124:F149)</f>
+        <f>SUMIF(E124:E149,"&gt;0",F124:F149)</f>
         <v/>
       </c>
       <c r="G150" s="24">
@@ -6924,7 +6947,7 @@
       <c r="C151" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D151" s="17" t="n">
+      <c r="D151" s="47" t="n">
         <v>77.81999999999999</v>
       </c>
       <c r="E151" s="18" t="n">
@@ -6964,7 +6987,7 @@
       <c r="C152" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D152" s="17" t="n">
+      <c r="D152" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E152" s="18" t="n">
@@ -7004,7 +7027,7 @@
       <c r="C153" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D153" s="17" t="n">
+      <c r="D153" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E153" s="18" t="n">
@@ -7044,7 +7067,7 @@
       <c r="C154" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D154" s="17" t="n">
+      <c r="D154" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E154" s="18" t="n">
@@ -7084,7 +7107,7 @@
       <c r="C155" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D155" s="17" t="n">
+      <c r="D155" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E155" s="18" t="n">
@@ -7124,7 +7147,7 @@
       <c r="C156" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D156" s="17" t="n">
+      <c r="D156" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E156" s="18" t="n">
@@ -7164,7 +7187,7 @@
       <c r="C157" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D157" s="17" t="n">
+      <c r="D157" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E157" s="18" t="n">
@@ -7204,7 +7227,7 @@
       <c r="C158" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D158" s="17" t="n">
+      <c r="D158" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E158" s="18" t="n">
@@ -7244,7 +7267,7 @@
       <c r="C159" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D159" s="17" t="n">
+      <c r="D159" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E159" s="18" t="n">
@@ -7284,7 +7307,7 @@
       <c r="C160" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D160" s="17" t="n">
+      <c r="D160" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E160" s="18" t="n">
@@ -7324,7 +7347,7 @@
       <c r="C161" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D161" s="17" t="n">
+      <c r="D161" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E161" s="18" t="n">
@@ -7364,7 +7387,7 @@
       <c r="C162" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D162" s="17" t="n">
+      <c r="D162" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E162" s="18" t="n">
@@ -7404,7 +7427,7 @@
       <c r="C163" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D163" s="17" t="n">
+      <c r="D163" s="47" t="n">
         <v>77.81</v>
       </c>
       <c r="E163" s="18" t="n">
@@ -7444,7 +7467,7 @@
       <c r="C164" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D164" s="17" t="n">
+      <c r="D164" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E164" s="18" t="n">
@@ -7484,7 +7507,7 @@
       <c r="C165" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D165" s="17" t="n">
+      <c r="D165" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E165" s="18" t="n">
@@ -7524,7 +7547,7 @@
       <c r="C166" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D166" s="17" t="n">
+      <c r="D166" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E166" s="18" t="n">
@@ -7564,7 +7587,7 @@
       <c r="C167" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D167" s="17" t="n">
+      <c r="D167" s="47" t="n">
         <v>16.77</v>
       </c>
       <c r="E167" s="18" t="n">
@@ -7604,7 +7627,7 @@
       <c r="C168" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D168" s="17" t="n">
+      <c r="D168" s="47" t="n">
         <v>77.65000000000001</v>
       </c>
       <c r="E168" s="18" t="n">
@@ -7644,7 +7667,7 @@
       <c r="C169" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D169" s="17" t="n">
+      <c r="D169" s="47" t="n">
         <v>77.70999999999999</v>
       </c>
       <c r="E169" s="18" t="n">
@@ -7684,7 +7707,7 @@
       <c r="C170" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D170" s="17" t="n">
+      <c r="D170" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E170" s="18" t="n">
@@ -7724,7 +7747,7 @@
       <c r="C171" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D171" s="17" t="n">
+      <c r="D171" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E171" s="18" t="n">
@@ -7764,7 +7787,7 @@
       <c r="C172" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D172" s="17" t="n">
+      <c r="D172" s="47" t="n">
         <v>77.67</v>
       </c>
       <c r="E172" s="18" t="n">
@@ -7804,7 +7827,7 @@
       <c r="C173" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D173" s="17" t="n">
+      <c r="D173" s="47" t="n">
         <v>77.69</v>
       </c>
       <c r="E173" s="18" t="n">
@@ -7844,7 +7867,7 @@
       <c r="C174" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D174" s="17" t="n">
+      <c r="D174" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E174" s="18" t="n">
@@ -7884,7 +7907,7 @@
       <c r="C175" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D175" s="17" t="n">
+      <c r="D175" s="47" t="n">
         <v>77.70999999999999</v>
       </c>
       <c r="E175" s="18" t="n">
@@ -7924,7 +7947,7 @@
       <c r="C176" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D176" s="17" t="n">
+      <c r="D176" s="47" t="n">
         <v>19.2</v>
       </c>
       <c r="E176" s="18" t="n">
@@ -7964,7 +7987,7 @@
       <c r="C177" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D177" s="17" t="n">
+      <c r="D177" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E177" s="18" t="n">
@@ -8004,7 +8027,7 @@
       <c r="C178" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D178" s="17" t="n">
+      <c r="D178" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E178" s="18" t="n">
@@ -8044,7 +8067,7 @@
       <c r="C179" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D179" s="17" t="n">
+      <c r="D179" s="47" t="n">
         <v>77.78</v>
       </c>
       <c r="E179" s="18" t="n">
@@ -8084,7 +8107,7 @@
       <c r="C180" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D180" s="17" t="n">
+      <c r="D180" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E180" s="18" t="n">
@@ -8124,7 +8147,7 @@
       <c r="C181" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D181" s="17" t="n">
+      <c r="D181" s="47" t="n">
         <v>77.36</v>
       </c>
       <c r="E181" s="18" t="n">
@@ -8164,7 +8187,7 @@
       <c r="C182" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D182" s="17" t="n">
+      <c r="D182" s="47" t="n">
         <v>77.79000000000001</v>
       </c>
       <c r="E182" s="18" t="n">
@@ -8204,7 +8227,7 @@
       <c r="C183" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D183" s="17" t="n">
+      <c r="D183" s="47" t="n">
         <v>72.3</v>
       </c>
       <c r="E183" s="18" t="n">
@@ -8244,7 +8267,7 @@
       <c r="C184" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D184" s="17" t="n">
+      <c r="D184" s="47" t="n">
         <v>32.16</v>
       </c>
       <c r="E184" s="18" t="n">
@@ -8284,7 +8307,7 @@
       <c r="C185" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D185" s="17" t="n">
+      <c r="D185" s="47" t="n">
         <v>16.38</v>
       </c>
       <c r="E185" s="18" t="n">
@@ -8325,7 +8348,7 @@
         <f>SUM(C151:C185)</f>
         <v/>
       </c>
-      <c r="D186" s="22">
+      <c r="D186" s="48">
         <f>SUM(D151:D185)</f>
         <v/>
       </c>
@@ -8334,7 +8357,7 @@
         <v/>
       </c>
       <c r="F186" s="23">
-        <f>SUM(F151:F185)</f>
+        <f>SUMIF(E151:E185,"&gt;0",F151:F185)</f>
         <v/>
       </c>
       <c r="G186" s="24">
@@ -8372,7 +8395,7 @@
       <c r="C187" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D187" s="17" t="n">
+      <c r="D187" s="47" t="n">
         <v>77.81999999999999</v>
       </c>
       <c r="E187" s="18" t="n">
@@ -8412,7 +8435,7 @@
       <c r="C188" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D188" s="17" t="n">
+      <c r="D188" s="47" t="n">
         <v>77.87</v>
       </c>
       <c r="E188" s="18" t="n">
@@ -8452,7 +8475,7 @@
       <c r="C189" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D189" s="17" t="n">
+      <c r="D189" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E189" s="18" t="n">
@@ -8492,7 +8515,7 @@
       <c r="C190" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D190" s="17" t="n">
+      <c r="D190" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E190" s="18" t="n">
@@ -8532,7 +8555,7 @@
       <c r="C191" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D191" s="17" t="n">
+      <c r="D191" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E191" s="18" t="n">
@@ -8572,7 +8595,7 @@
       <c r="C192" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D192" s="17" t="n">
+      <c r="D192" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E192" s="18" t="n">
@@ -8612,7 +8635,7 @@
       <c r="C193" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D193" s="17" t="n">
+      <c r="D193" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E193" s="18" t="n">
@@ -8652,7 +8675,7 @@
       <c r="C194" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D194" s="17" t="n">
+      <c r="D194" s="47" t="n">
         <v>77.59999999999999</v>
       </c>
       <c r="E194" s="18" t="n">
@@ -8692,7 +8715,7 @@
       <c r="C195" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D195" s="17" t="n">
+      <c r="D195" s="47" t="n">
         <v>77.73</v>
       </c>
       <c r="E195" s="18" t="n">
@@ -8732,7 +8755,7 @@
       <c r="C196" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D196" s="17" t="n">
+      <c r="D196" s="47" t="n">
         <v>12.84</v>
       </c>
       <c r="E196" s="18" t="n">
@@ -8772,7 +8795,7 @@
       <c r="C197" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D197" s="17" t="n">
+      <c r="D197" s="47" t="n">
         <v>77.59999999999999</v>
       </c>
       <c r="E197" s="18" t="n">
@@ -8812,7 +8835,7 @@
       <c r="C198" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D198" s="17" t="n">
+      <c r="D198" s="47" t="n">
         <v>77.86</v>
       </c>
       <c r="E198" s="18" t="n">
@@ -8852,7 +8875,7 @@
       <c r="C199" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D199" s="17" t="n">
+      <c r="D199" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E199" s="18" t="n">
@@ -8892,7 +8915,7 @@
       <c r="C200" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D200" s="17" t="n">
+      <c r="D200" s="47" t="n">
         <v>77.84</v>
       </c>
       <c r="E200" s="18" t="n">
@@ -8932,7 +8955,7 @@
       <c r="C201" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D201" s="17" t="n">
+      <c r="D201" s="47" t="n">
         <v>77.73999999999999</v>
       </c>
       <c r="E201" s="18" t="n">
@@ -8972,7 +8995,7 @@
       <c r="C202" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D202" s="17" t="n">
+      <c r="D202" s="47" t="n">
         <v>77.65000000000001</v>
       </c>
       <c r="E202" s="18" t="n">
@@ -9012,7 +9035,7 @@
       <c r="C203" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D203" s="17" t="n">
+      <c r="D203" s="47" t="n">
         <v>3.87</v>
       </c>
       <c r="E203" s="18" t="n">
@@ -9052,7 +9075,7 @@
       <c r="C204" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D204" s="17" t="n">
+      <c r="D204" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E204" s="18" t="n">
@@ -9092,7 +9115,7 @@
       <c r="C205" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D205" s="17" t="n">
+      <c r="D205" s="47" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E205" s="18" t="n">
@@ -9132,7 +9155,7 @@
       <c r="C206" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D206" s="17" t="n">
+      <c r="D206" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E206" s="18" t="n">
@@ -9172,7 +9195,7 @@
       <c r="C207" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D207" s="17" t="n">
+      <c r="D207" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E207" s="18" t="n">
@@ -9212,7 +9235,7 @@
       <c r="C208" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D208" s="17" t="n">
+      <c r="D208" s="47" t="n">
         <v>77.81999999999999</v>
       </c>
       <c r="E208" s="18" t="n">
@@ -9252,7 +9275,7 @@
       <c r="C209" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D209" s="17" t="n">
+      <c r="D209" s="47" t="n">
         <v>77.72</v>
       </c>
       <c r="E209" s="18" t="n">
@@ -9292,7 +9315,7 @@
       <c r="C210" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D210" s="17" t="n">
+      <c r="D210" s="47" t="n">
         <v>77.66</v>
       </c>
       <c r="E210" s="18" t="n">
@@ -9332,7 +9355,7 @@
       <c r="C211" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D211" s="17" t="n">
+      <c r="D211" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E211" s="18" t="n">
@@ -9372,7 +9395,7 @@
       <c r="C212" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D212" s="17" t="n">
+      <c r="D212" s="47" t="n">
         <v>77.67</v>
       </c>
       <c r="E212" s="18" t="n">
@@ -9412,7 +9435,7 @@
       <c r="C213" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D213" s="17" t="n">
+      <c r="D213" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E213" s="18" t="n">
@@ -9452,7 +9475,7 @@
       <c r="C214" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D214" s="17" t="n">
+      <c r="D214" s="47" t="n">
         <v>68.09</v>
       </c>
       <c r="E214" s="18" t="n">
@@ -9492,7 +9515,7 @@
       <c r="C215" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D215" s="17" t="n">
+      <c r="D215" s="47" t="n">
         <v>51.07</v>
       </c>
       <c r="E215" s="18" t="n">
@@ -9532,7 +9555,7 @@
       <c r="C216" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D216" s="17" t="n">
+      <c r="D216" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E216" s="18" t="n">
@@ -9572,7 +9595,7 @@
       <c r="C217" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D217" s="17" t="n">
+      <c r="D217" s="47" t="n">
         <v>77.7</v>
       </c>
       <c r="E217" s="18" t="n">
@@ -9612,7 +9635,7 @@
       <c r="C218" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D218" s="17" t="n">
+      <c r="D218" s="47" t="n">
         <v>77.83</v>
       </c>
       <c r="E218" s="18" t="n">
@@ -9652,7 +9675,7 @@
       <c r="C219" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D219" s="17" t="n">
+      <c r="D219" s="47" t="n">
         <v>20.14</v>
       </c>
       <c r="E219" s="18" t="n">
@@ -9692,7 +9715,7 @@
       <c r="C220" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D220" s="17" t="n">
+      <c r="D220" s="47" t="n">
         <v>0</v>
       </c>
       <c r="E220" s="18" t="n">
@@ -9733,7 +9756,7 @@
         <f>SUM(C187:C220)</f>
         <v/>
       </c>
-      <c r="D221" s="22">
+      <c r="D221" s="48">
         <f>SUM(D187:D220)</f>
         <v/>
       </c>
@@ -9742,7 +9765,7 @@
         <v/>
       </c>
       <c r="F221" s="23">
-        <f>SUM(F187:F220)</f>
+        <f>SUMIF(E187:E220,"&gt;0",F187:F220)</f>
         <v/>
       </c>
       <c r="G221" s="24">
@@ -9777,7 +9800,7 @@
         <f>C35+C65+C95+C123+C150+C186+C221</f>
         <v/>
       </c>
-      <c r="D222" s="27">
+      <c r="D222" s="49">
         <f>D35+D65+D95+D123+D150+D186+D221</f>
         <v/>
       </c>
@@ -9853,7 +9876,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="30" t="inlineStr">
         <is>
@@ -9861,7 +9883,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -10469,7 +10490,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -21792,7 +21812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="B1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -21807,7 +21827,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="B3" s="42" t="inlineStr">
         <is>

</xml_diff>